<commit_message>
Ferramenta 8: Imagem de Fundo (1.1.0)
Baixa imagem de satélite ou de mapa (serviços da Esri) no sistema de
coordenadas da rede, grava em BMP e escreve a seção [BACKDROP] para o
fundo aparecer alinhado no EPANET 2.2 Brasil. Manual, LEIA-ME, planilha
e CHANGELOG atualizados.
</commit_message>
<xml_diff>
--- a/epanet_br_tools/Cadastro_Ferramentas_EPANET_Br.xlsx
+++ b/epanet_br_tools/Cadastro_Ferramentas_EPANET_Br.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="13" min="1" max="1"/>
@@ -971,57 +971,102 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="27.75" customHeight="1" s="14"/>
-    <row r="22" ht="27.75" customHeight="1" s="14">
-      <c r="A22" s="24" t="inlineStr">
+    <row r="21" ht="45.75" customHeight="1" s="14">
+      <c r="A21" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>Imagem de Fundo</t>
+        </is>
+      </c>
+      <c r="C21" s="22">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="D21" s="22">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E21" s="22">
+        <f>""""&amp;$B$6&amp;"\08_imagem_fundo.py"" $INPFILE"</f>
+        <v/>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t>Baixa imagem de satélite ou de mapa no sistema de coordenadas da rede e grava o fundo ([BACKDROP]) já alinhado. Precisa de internet e rede georreferenciada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="27.75" customHeight="1" s="14"/>
+    <row r="23" ht="27.75" customHeight="1" s="14">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Observações</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="27.75" customHeight="1" s="14">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>• O campo Programa é sempre o pythonw.exe, nunca o .py. Apontar para o .py faz o Windows abrir o arquivo no VS Code.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="27.75" customHeight="1" s="14">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>• Para ver erros na primeira vez, troque pythonw.exe por python.exe no campo Programa (abre uma janela preta com as mensagens).</t>
+          <t>• O campo Programa é sempre o pythonw.exe, nunca o .py. Apontar para o .py faz o Windows abrir o arquivo no VS Code.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="27.75" customHeight="1" s="14">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>• As ferramentas 4 e 5 procuram o runepanet.exe em C:\Program Files (x86)\Epanet 2.2 Brasil. Se o EPANET Br estiver em outro lugar, copie o runepanet.exe para a pasta das ferramentas.</t>
+          <t>• Para ver erros na primeira vez, troque pythonw.exe por python.exe no campo Programa (abre uma janela preta com as mensagens).</t>
         </is>
       </c>
     </row>
     <row r="26" ht="27.75" customHeight="1" s="14">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>• O EPANET 2.2 Brasil não oferece $OUTFILE; por isso todas as ferramentas recebem só $INPFILE.</t>
+          <t>• As ferramentas 4 e 5 procuram o runepanet.exe em C:\Program Files (x86)\Epanet 2.2 Brasil. Se o EPANET Br estiver em outro lugar, copie o runepanet.exe para a pasta das ferramentas.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="27.75" customHeight="1" s="14">
       <c r="A27" s="25" t="inlineStr">
         <is>
+          <t>• O EPANET 2.2 Brasil não oferece $OUTFILE; por isso todas as ferramentas recebem só $INPFILE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="27.75" customHeight="1" s="14">
+      <c r="A28" s="25" t="inlineStr">
+        <is>
           <t>• Se aparecer 'I/O error 32' ao salvar, feche todas as janelas de EPANET (inclusive outras versões) e cadastre de novo.</t>
         </is>
       </c>
     </row>
+    <row r="29" ht="27.75" customHeight="1" s="14">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>• A ferramenta 8 precisa de internet (services.arcgisonline.com). Atrás de proxy, peça a liberação à TI.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A29:H29"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>